<commit_message>
Schools datasets + Leaflet maps for all ebarilga choropleths
- Add ebarilga-schools (323-school directory) and ebarilga-schools-by-khoroo
  (per-khoroo counts) as bilingual datasets with counts/directory builders
- New MapChart component: Leaflet pan/zoom choropleths that read the Vega
  spec file as config; migrate all 5 ebarilga map datasets (EN+MN) with
  wide layout, Reset control, and plain-text attribution
- Register schools in reference-table pipeline; validator accepts MapChart
- Transliteration: acronym-caps rule + EN/DE-origin exception names
</commit_message>
<xml_diff>
--- a/data.mn/public/datasets/ebarilga-zip-zones.xlsx
+++ b/data.mn/public/datasets/ebarilga-zip-zones.xlsx
@@ -1570,7 +1570,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Zamchin-BKhD</t>
+          <t>Zamchin-BKD</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -14233,7 +14233,7 @@
       </c>
       <c r="B512" t="inlineStr">
         <is>
-          <t>Khundlungiin am-SKhD</t>
+          <t>Khundlungiin am-SKD</t>
         </is>
       </c>
       <c r="C512" t="n">

</xml_diff>